<commit_message>
was updated the process using the LLM's
</commit_message>
<xml_diff>
--- a/tabla_estudios.xlsx
+++ b/tabla_estudios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/d_agudelo_cgiar_org/Documents/Desktop/diet_project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/d_agudelo_cgiar_org/Documents/Desktop/codigos_dengue/diet_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7D8EC97-7FA6-4C25-AF6F-DEB834EB9BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{C7D8EC97-7FA6-4C25-AF6F-DEB834EB9BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC4865CF-4FD0-4C2B-9604-E839FBB323A5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{22204672-031F-436F-B8C7-A470BDA11F1F}"/>
   </bookViews>
@@ -724,6 +724,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC3E7283-2B43-43BC-BC64-48FD451EB534}">
   <dimension ref="A1:AB13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="191.85546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>